<commit_message>
fix(downloads): prevent 404 text downloads by adding on_click='ignore' and pinning session
</commit_message>
<xml_diff>
--- a/data/sync_databases/BD_Datos_Generales_Remision.xlsx
+++ b/data/sync_databases/BD_Datos_Generales_Remision.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H108"/>
+  <dimension ref="A1:H146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4484,11 +4484,11 @@
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>E0132</t>
+          <t>E0133</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -4508,32 +4508,32 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>EQM</t>
+          <t>PLANTA RIO XIX</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Calle Inde 714, 35079 Gómez Palacio, Durango</t>
+          <t>Carlos Salinas de Gortari 43, Nueva Laguna Nte., 27110 Torreón, Coah.</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>['TPM-0522', 'TPM-0456', 'TPM-0444', 'TPM-0326', 'TPM-0500', 'TPM-0211']</t>
+          <t>['TPM-0523']</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>E0133</t>
+          <t>E0134</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>01/09/2026</t>
+          <t>04/09/2026</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -4558,22 +4558,22 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>['TPM-0523']</t>
+          <t>['TPM-0524', 'TPM-0539', 'TPM-0525', 'TPM-0526', 'TPM-0540']</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>E0134</t>
+          <t>E0135</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>04/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -4588,32 +4588,32 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>PLANTA RIO XIX</t>
+          <t>EQM</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Carlos Salinas de Gortari 43, Nueva Laguna Nte., 27110 Torreón, Coah.</t>
+          <t>Calle Inde 714, 35079 Gómez Palacio, Durango</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>['TPM-0524', 'TPM-0539', 'TPM-0525', 'TPM-0526', 'TPM-0540']</t>
+          <t>['TPM-0547', 'TPM-0546', 'TPM-0545', 'TPM-0544', 'TPM-0543', 'TPM-0542']</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>E0135</t>
+          <t>E0136</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>10/09/2026</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -4638,7 +4638,1527 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>['TPM-0547', 'TPM-0546', 'TPM-0545', 'TPM-0544', 'TPM-0543', 'TPM-0542']</t>
+          <t>['TPM-0556']</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>111</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>E0137</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Carlos Salinas de Gortari 43, Nueva Laguna Nte., 27110 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>['TPM-0566', 'TPM-0565', 'TPM-0564', 'TPM-0563', 'TPM-0562', 'TPM-0561']</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>112</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>E0138</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>['TPM-0480', 'TPM-0481', 'TPM-0482']</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>113</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>E0139</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>['TPM-0476', 'TPM-0474', 'TPM-0477', 'TPM-0475', 'TPM-0479', 'TPM-0478']</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>114</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>E0140</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>['TPM-0533', 'TPM-0538', 'TPM-0536', 'TPM-0537', 'TPM-0532', 'TPM-0535', 'TPM-0528', 'TPM-0531', 'TPM-0530', 'TPM-0534', 'TPM-0529', 'TPM-0470', 'TPM-0471', 'TPM-0473', 'TPM-0450', 'TPM-0451', 'TPM-0449', 'TPM-0469', 'TPM-0527']</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>115</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>E0141</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>['TPM-0306', 'TPM-0454', 'TPM-0455']</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>116</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>E0142</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>['TPM-0548', 'TPM-0448', 'TPM-0453', 'TPM-0457', 'TPM-0483', 'TPM-0460']</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>117</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>E0143</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>21/09/2026</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>['TPM-0550', 'TPM-0551', 'TPM-0552', 'TPM-0485', 'TPM-0549', 'TPM-0458', 'TPM-0484']</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>118</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>E0144</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>21/09/2026</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>['TPM-0555', 'TPM-0554', 'TPM-0553']</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>119</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>E0145</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>21/09/2026</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>['TPM-0472', 'TPM-0541', 'TPM-0452']</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>120</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>E0146</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>['TPM-0576']</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>121</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>E0147</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Carlos Salinas de Gortari 43, Nueva Laguna Nte., 27110 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>['TPM-0567', 'TPM-0568', 'TPM-0575']</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>122</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>E0148</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Carlos Salinas de Gortari 43, Nueva Laguna Nte., 27110 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>['TPM-0579', 'TPM-0578', 'TPM-0577']</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>123</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>E0149</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Calle Inde 714, 35079 Gómez Palacio, Durango</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>['TPM-0580']</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>124</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>E0150</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Calle Inde 714, 35079 Gómez Palacio, Durango</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>['TPM-0581']</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>125</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>E0151</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Calle Inde 714, 35079 Gómez Palacio, Durango</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>['TPM-0558']</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>127</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>E0153</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Carlos Salinas de Gortari 43, Nueva Laguna Nte., 27110 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>['TPM-0559']</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>128</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>E0154</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Carlos Salinas de Gortari 43, Nueva Laguna Nte., 27110 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>['TPM-0584', 'TPM-0585']</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>129</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>E0155</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Carlos Salinas de Gortari 43, Nueva Laguna Nte., 27110 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>['TPM-0589', 'TPM-0588', 'TPM-0587', 'TPM-0586']</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>130</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>E0156</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Carlos Salinas de Gortari 43, Nueva Laguna Nte., 27110 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>['TPM-0592', 'TPM-0591', 'TPM-0590']</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>131</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>E0157</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>EQM</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Calle Inde 714, 35079 Gómez Palacio, Durango</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>['TPM-0621']</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>132</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>E0158</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Carlos Salinas de Gortari 43, Nueva Laguna Nte., 27110 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>['TPM-0620']</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>133</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>E0159</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>['TPM-0582', 'TPM-0616', 'TPM-0617', 'TPM-0618', 'TPM-0619', 'TPM-0634']</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>134</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>E0160</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>['TPM-0635', 'TPM-0633']</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>135</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>E0161</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>['TPM-0211', 'TPM-0326', 'TPM-0444', 'TPM-0456', 'TPM-0500', 'TPM-0593']</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>136</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>E0162</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>['TPM-0594', 'TPM-0595', 'TPM-0596']</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>137</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>E0163</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>['TPM-0599', 'TPM-0603', 'TPM-0604', 'TPM-0605', 'TPM-0611', 'TPM-0613']</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>138</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>E0164</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>['TPM-0598', 'TPM-0608', 'TPM-0601']</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>139</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>E0165</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>['TPM-0602', 'TPM-0606', 'TPM-0609', 'TPM-0612', 'TPM-0614', 'TPM-0615']</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>140</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>E0166</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>['TPM-0569', 'TPM-0570', 'TPM-0571']</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>141</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>E0167</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>['TPM-0572', 'TPM-0597', 'TPM-0600', 'TPM-0607', 'TPM-0610']</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>142</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>E0168</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>['TPM-0574', 'TPM-0636']</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>143</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>E0169</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>['TPM-0522']</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>144</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>E0170</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Carlos Salinas de Gortari 43, Nueva Laguna Nte., 27110 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>['TPM-0658', 'TPM-0659', 'TPM-0660']</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>145</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>E0171</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Carlos Salinas de Gortari 43, Nueva Laguna Nte., 27110 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>['TPM-0646', 'TPM-0647']</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>146</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>E0172</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Carlos Salinas de Gortari 43, Nueva Laguna Nte., 27110 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>['TPM-0649']</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>147</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>E0173</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>14/10/2026</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Galvatec Industrias</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Prol. Valle Guadiana 919, Parque Industrial II, 35078 Gómez Palacio, Dgo.</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>['TPM-0557']</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>148</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>E0174</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>14/10/2026</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>kirbymex</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Carretera Torreón, Blvr. Mieleras 163 Ote, Sta Sofía, 27293 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>['TPM-0648', 'TPM-0680', 'TPM-0583']</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>149</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>E0175</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Metales</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>PLANTA RIO XIX</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Carlos Salinas de Gortari 43, Nueva Laguna Nte., 27110 Torreón, Coah.</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>['TPM-0686']</t>
         </is>
       </c>
     </row>

</xml_diff>